<commit_message>
Changes to step 6
</commit_message>
<xml_diff>
--- a/M1000-100_data.xlsx
+++ b/M1000-100_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dtudk-my.sharepoint.com/personal/nemi_dtu_dk/Documents/M/3_Lector/01_Teaching/46725/24/1_Ass/Design/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willi\OneDrive\Skrivebord\DTU\2. Electrical Machines\Assignment 1\Assignment_1_electrical_machines\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_2626D058230C65E4840604F6E457F0BE37C6FB86" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3196F53-8140-4992-82E3-A68E580246FD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C90CCCE5-23E5-4494-BFF7-331EFBDE3AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="79200" yWindow="2190" windowWidth="16725" windowHeight="16515" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -234,6 +234,2147 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="da-DK"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="da-DK"/>
+              <a:t>M1000-100</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="da-DK"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="log"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="da-DK"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$5:$A$203</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="199"/>
+                <c:pt idx="0">
+                  <c:v>6.8671679320000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>13.05931629</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>18.550231419999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>23.4909325</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>27.986195899999998</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>32.116098409999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>35.941569080000001</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>39.509859179999999</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>42.858295310000003</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>46.016877360000002</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>49.010094979999998</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>51.8582204</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>54.578245819999999</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>57.184575760000001</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>59.68954695</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>62.10382508</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>64.436711790000004</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>66.696385500000005</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>68.89009265</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>71.024301269999995</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>73.10482571</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>75.13692897</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>77.125407510000002</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>79.074662200000006</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>80.988758379999993</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>82.871477060000004</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>84.726359160000001</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>86.556744080000001</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>88.365803830000004</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>90.156573429999995</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>91.931978580000006</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>93.694861029999998</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>95.448002320000001</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>97.194146329999995</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>98.936020979999995</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>100.6763596</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>102.4179221</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>104.16351659999999</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>105.9160217</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>107.6784092</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>109.4537684</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>111.2453318</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>113.05650249999999</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>114.890883</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>116.752307</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>118.64487219999999</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>120.5729759</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>122.54185200000001</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>124.5896113</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>126.7346713</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>128.98503880000001</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>131.34940180000001</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>133.83751520000001</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>136.4603764</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>139.2304245</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>142.16177329999999</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>145.27047970000001</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>148.5748523</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>152.0957946</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>155.8571772</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>159.88621560000001</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>164.2138118</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>168.87478369999999</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>173.90785500000001</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>179.35520729999999</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>185.26131860000001</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>191.67074589999999</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>198.62454410000001</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>206.15524479999999</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>214.28088579999999</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>222.999425</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>232.2856074</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>242.09221479999999</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>252.35615870000001</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>263.00770269999998</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>273.97977300000002</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>285.2147683</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>296.66790630000003</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>308.30761890000002</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>320.11414000000002</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>332.07734420000003</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>344.19452960000001</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>356.4684853</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>368.9059537</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>381.5164734</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>394.31154479999998</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>407.30404549999997</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>420.50783389999998</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>433.93749050000002</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>447.60815580000002</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>461.53543960000002</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>475.73537870000001</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>490.22443070000003</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>505.0194932</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>520.13794180000002</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>535.59768250000002</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>551.41721600000005</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>567.61571140000001</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>584.21308929999998</c:v>
+                </c:pt>
+                <c:pt idx="99">
+                  <c:v>601.23011359999998</c:v>
+                </c:pt>
+                <c:pt idx="100">
+                  <c:v>618.68849230000001</c:v>
+                </c:pt>
+                <c:pt idx="101">
+                  <c:v>636.61098800000002</c:v>
+                </c:pt>
+                <c:pt idx="102">
+                  <c:v>655.02153920000001</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>673.94539320000001</c:v>
+                </c:pt>
+                <c:pt idx="104">
+                  <c:v>693.4092531</c:v>
+                </c:pt>
+                <c:pt idx="105">
+                  <c:v>713.44144019999999</c:v>
+                </c:pt>
+                <c:pt idx="106">
+                  <c:v>734.07207370000003</c:v>
+                </c:pt>
+                <c:pt idx="107">
+                  <c:v>755.33327199999997</c:v>
+                </c:pt>
+                <c:pt idx="108">
+                  <c:v>777.25937720000002</c:v>
+                </c:pt>
+                <c:pt idx="109">
+                  <c:v>799.88720709999996</c:v>
+                </c:pt>
+                <c:pt idx="110">
+                  <c:v>823.25634049999996</c:v>
+                </c:pt>
+                <c:pt idx="111">
+                  <c:v>847.4094384</c:v>
+                </c:pt>
+                <c:pt idx="112">
+                  <c:v>872.39261080000006</c:v>
+                </c:pt>
+                <c:pt idx="113">
+                  <c:v>898.25583410000002</c:v>
+                </c:pt>
+                <c:pt idx="114">
+                  <c:v>925.05342910000002</c:v>
+                </c:pt>
+                <c:pt idx="115">
+                  <c:v>952.84461229999999</c:v>
+                </c:pt>
+                <c:pt idx="116">
+                  <c:v>981.69413059999999</c:v>
+                </c:pt>
+                <c:pt idx="117">
+                  <c:v>1011.672999</c:v>
+                </c:pt>
+                <c:pt idx="118">
+                  <c:v>1042.859361</c:v>
+                </c:pt>
+                <c:pt idx="119">
+                  <c:v>1075.3394949999999</c:v>
+                </c:pt>
+                <c:pt idx="120">
+                  <c:v>1109.208995</c:v>
+                </c:pt>
+                <c:pt idx="121">
+                  <c:v>1144.574179</c:v>
+                </c:pt>
+                <c:pt idx="122">
+                  <c:v>1181.55375</c:v>
+                </c:pt>
+                <c:pt idx="123">
+                  <c:v>1220.280796</c:v>
+                </c:pt>
+                <c:pt idx="124">
+                  <c:v>1260.905188</c:v>
+                </c:pt>
+                <c:pt idx="125">
+                  <c:v>1303.5964959999999</c:v>
+                </c:pt>
+                <c:pt idx="126">
+                  <c:v>1348.54755</c:v>
+                </c:pt>
+                <c:pt idx="127">
+                  <c:v>1395.9788100000001</c:v>
+                </c:pt>
+                <c:pt idx="128">
+                  <c:v>1446.1438089999999</c:v>
+                </c:pt>
+                <c:pt idx="129">
+                  <c:v>1499.3359479999999</c:v>
+                </c:pt>
+                <c:pt idx="130">
+                  <c:v>1555.8971039999999</c:v>
+                </c:pt>
+                <c:pt idx="131">
+                  <c:v>1616.228625</c:v>
+                </c:pt>
+                <c:pt idx="132">
+                  <c:v>1680.805537</c:v>
+                </c:pt>
+                <c:pt idx="133">
+                  <c:v>1750.1951570000001</c:v>
+                </c:pt>
+                <c:pt idx="134">
+                  <c:v>1825.0817930000001</c:v>
+                </c:pt>
+                <c:pt idx="135">
+                  <c:v>1906.3000460000001</c:v>
+                </c:pt>
+                <c:pt idx="136">
+                  <c:v>1994.8804689999999</c:v>
+                </c:pt>
+                <c:pt idx="137">
+                  <c:v>2092.1133540000001</c:v>
+                </c:pt>
+                <c:pt idx="138">
+                  <c:v>2199.6397459999998</c:v>
+                </c:pt>
+                <c:pt idx="139">
+                  <c:v>2319.5843589999999</c:v>
+                </c:pt>
+                <c:pt idx="140">
+                  <c:v>2454.75486</c:v>
+                </c:pt>
+                <c:pt idx="141">
+                  <c:v>2608.9495069999998</c:v>
+                </c:pt>
+                <c:pt idx="142">
+                  <c:v>2787.4477310000002</c:v>
+                </c:pt>
+                <c:pt idx="143">
+                  <c:v>2997.820471</c:v>
+                </c:pt>
+                <c:pt idx="144">
+                  <c:v>3251.318327</c:v>
+                </c:pt>
+                <c:pt idx="145">
+                  <c:v>3565.3275440000002</c:v>
+                </c:pt>
+                <c:pt idx="146">
+                  <c:v>3967.7694329999999</c:v>
+                </c:pt>
+                <c:pt idx="147">
+                  <c:v>4504.5108710000004</c:v>
+                </c:pt>
+                <c:pt idx="148">
+                  <c:v>5247.5704539999997</c:v>
+                </c:pt>
+                <c:pt idx="149">
+                  <c:v>6279.0885420000004</c:v>
+                </c:pt>
+                <c:pt idx="150">
+                  <c:v>7581.555816</c:v>
+                </c:pt>
+                <c:pt idx="151">
+                  <c:v>8963.1991959999996</c:v>
+                </c:pt>
+                <c:pt idx="152">
+                  <c:v>10290.372460000001</c:v>
+                </c:pt>
+                <c:pt idx="153">
+                  <c:v>11547.06855</c:v>
+                </c:pt>
+                <c:pt idx="154">
+                  <c:v>12747.270490000001</c:v>
+                </c:pt>
+                <c:pt idx="155">
+                  <c:v>13907.195900000001</c:v>
+                </c:pt>
+                <c:pt idx="156">
+                  <c:v>15040.515219999999</c:v>
+                </c:pt>
+                <c:pt idx="157">
+                  <c:v>16158.14286</c:v>
+                </c:pt>
+                <c:pt idx="158">
+                  <c:v>17268.83959</c:v>
+                </c:pt>
+                <c:pt idx="159">
+                  <c:v>18379.815689999999</c:v>
+                </c:pt>
+                <c:pt idx="160">
+                  <c:v>19497.199700000001</c:v>
+                </c:pt>
+                <c:pt idx="161">
+                  <c:v>20626.38334</c:v>
+                </c:pt>
+                <c:pt idx="162">
+                  <c:v>21772.275300000001</c:v>
+                </c:pt>
+                <c:pt idx="163">
+                  <c:v>22939.492969999999</c:v>
+                </c:pt>
+                <c:pt idx="164">
+                  <c:v>24132.51296</c:v>
+                </c:pt>
+                <c:pt idx="165">
+                  <c:v>25355.795620000001</c:v>
+                </c:pt>
+                <c:pt idx="166">
+                  <c:v>26613.894390000001</c:v>
+                </c:pt>
+                <c:pt idx="167">
+                  <c:v>27911.557980000001</c:v>
+                </c:pt>
+                <c:pt idx="168">
+                  <c:v>29253.832170000001</c:v>
+                </c:pt>
+                <c:pt idx="169">
+                  <c:v>30646.166949999999</c:v>
+                </c:pt>
+                <c:pt idx="170">
+                  <c:v>32094.535100000001</c:v>
+                </c:pt>
+                <c:pt idx="171">
+                  <c:v>33605.568429999999</c:v>
+                </c:pt>
+                <c:pt idx="172">
+                  <c:v>35186.719559999998</c:v>
+                </c:pt>
+                <c:pt idx="173">
+                  <c:v>36846.459000000003</c:v>
+                </c:pt>
+                <c:pt idx="174">
+                  <c:v>38594.520369999998</c:v>
+                </c:pt>
+                <c:pt idx="175">
+                  <c:v>40442.211640000001</c:v>
+                </c:pt>
+                <c:pt idx="176">
+                  <c:v>42402.817309999999</c:v>
+                </c:pt>
+                <c:pt idx="177">
+                  <c:v>44492.127489999999</c:v>
+                </c:pt>
+                <c:pt idx="178">
+                  <c:v>46729.14718</c:v>
+                </c:pt>
+                <c:pt idx="179">
+                  <c:v>49137.066489999997</c:v>
+                </c:pt>
+                <c:pt idx="180">
+                  <c:v>51744.617610000001</c:v>
+                </c:pt>
+                <c:pt idx="181">
+                  <c:v>54588.021309999996</c:v>
+                </c:pt>
+                <c:pt idx="182">
+                  <c:v>57713.861089999999</c:v>
+                </c:pt>
+                <c:pt idx="183">
+                  <c:v>61183.473890000001</c:v>
+                </c:pt>
+                <c:pt idx="184">
+                  <c:v>65079.934569999998</c:v>
+                </c:pt>
+                <c:pt idx="185">
+                  <c:v>69519.727209999997</c:v>
+                </c:pt>
+                <c:pt idx="186">
+                  <c:v>74673.481299999999</c:v>
+                </c:pt>
+                <c:pt idx="187">
+                  <c:v>80805.828429999994</c:v>
+                </c:pt>
+                <c:pt idx="188">
+                  <c:v>88360.487080000006</c:v>
+                </c:pt>
+                <c:pt idx="189">
+                  <c:v>98170.869470000005</c:v>
+                </c:pt>
+                <c:pt idx="190">
+                  <c:v>112114.4518</c:v>
+                </c:pt>
+                <c:pt idx="191">
+                  <c:v>134675.64189999999</c:v>
+                </c:pt>
+                <c:pt idx="192">
+                  <c:v>171180.41440000001</c:v>
+                </c:pt>
+                <c:pt idx="193">
+                  <c:v>230246.37710000001</c:v>
+                </c:pt>
+                <c:pt idx="194">
+                  <c:v>284156.97989999998</c:v>
+                </c:pt>
+                <c:pt idx="195">
+                  <c:v>332357.217</c:v>
+                </c:pt>
+                <c:pt idx="196">
+                  <c:v>379288.90899999999</c:v>
+                </c:pt>
+                <c:pt idx="197">
+                  <c:v>426314.05430000002</c:v>
+                </c:pt>
+                <c:pt idx="198">
+                  <c:v>474144.42190000002</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$B$5:$B$203</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="199"/>
+                <c:pt idx="0">
+                  <c:v>1.0177903E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.0123520999999998E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.9615546E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.8747012999999997E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.7581423999999997E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.6172489999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6.4563021999999998E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7.2787466999999995E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8.0873924999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>8.8845673E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>9.6722297999999998E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.10452052100000001</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.112254822</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.119937907</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.127581061</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.135194433</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.14278725</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.150367995</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.15794454499999999</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.16552429299999999</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.173114241</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.18072108200000001</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.18835126799999999</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.19601107800000001</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.20370666000000001</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.21144409</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.21922940699999999</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.22706865600000001</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.23496792499999999</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.242933383</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.25097130699999998</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>0.259088123</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>0.26729043099999999</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>0.27558504299999997</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>0.28397901199999998</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>0.292479661</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>0.30109462100000001</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>0.30983185400000002</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>0.31869969100000001</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>0.32770685500000002</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>0.33686248800000002</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>0.346176176</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>0.35565796700000002</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>0.36531837499999997</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>0.37516838000000002</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>0.38521940700000001</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>0.39548328500000002</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>0.40597488100000001</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>0.416886439</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>0.42831081100000001</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>0.44028475099999997</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>0.45284696099999999</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>0.46603971900000002</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>0.479909266</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>0.49450617000000002</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>0.50988568199999995</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>0.52610802599999995</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>0.54323859100000005</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>0.56134790400000001</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>0.58051124600000004</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>0.60080768500000004</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>0.62231818900000002</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>0.64512235699999998</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>0.66929312799999996</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>0.69488874</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>0.72194119199999995</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>0.75044085999999999</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>0.78031795699999995</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>0.81142355499999996</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>0.84351564000000001</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>0.876257968</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>0.90923870799999995</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>0.94200986799999997</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>0.97413885899999997</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>1.0052565579999999</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>1.035087782</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>1.06345917</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>1.0902888770000001</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>1.1155667789999999</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>1.139332893</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>1.1616585880000001</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>1.182632218</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>1.202349114</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>1.2209050960000001</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>1.23839258</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>1.25489845</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>1.270503079</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>1.285280054</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>1.2992963239999999</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>1.3126125790000001</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>1.3252837289999999</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>1.33735943</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>1.348884607</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>1.3598999460000001</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>1.37044235</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>1.3805453519999999</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>1.3902394890000001</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>1.399552632</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>1.4085102810000001</c:v>
+                </c:pt>
+                <c:pt idx="99">
+                  <c:v>1.417135824</c:v>
+                </c:pt>
+                <c:pt idx="100">
+                  <c:v>1.4254507679999999</c:v>
+                </c:pt>
+                <c:pt idx="101">
+                  <c:v>1.4334749419999999</c:v>
+                </c:pt>
+                <c:pt idx="102">
+                  <c:v>1.441226678</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>1.4487229690000001</c:v>
+                </c:pt>
+                <c:pt idx="104">
+                  <c:v>1.4559796119999999</c:v>
+                </c:pt>
+                <c:pt idx="105">
+                  <c:v>1.463011337</c:v>
+                </c:pt>
+                <c:pt idx="106">
+                  <c:v>1.469831917</c:v>
+                </c:pt>
+                <c:pt idx="107">
+                  <c:v>1.4764542679999999</c:v>
+                </c:pt>
+                <c:pt idx="108">
+                  <c:v>1.482890547</c:v>
+                </c:pt>
+                <c:pt idx="109">
+                  <c:v>1.48915223</c:v>
+                </c:pt>
+                <c:pt idx="110">
+                  <c:v>1.4952501890000001</c:v>
+                </c:pt>
+                <c:pt idx="111">
+                  <c:v>1.501194763</c:v>
+                </c:pt>
+                <c:pt idx="112">
+                  <c:v>1.5069958219999999</c:v>
+                </c:pt>
+                <c:pt idx="113">
+                  <c:v>1.51266283</c:v>
+                </c:pt>
+                <c:pt idx="114">
+                  <c:v>1.5182048990000001</c:v>
+                </c:pt>
+                <c:pt idx="115">
+                  <c:v>1.523630848</c:v>
+                </c:pt>
+                <c:pt idx="116">
+                  <c:v>1.528949256</c:v>
+                </c:pt>
+                <c:pt idx="117">
+                  <c:v>1.534168515</c:v>
+                </c:pt>
+                <c:pt idx="118">
+                  <c:v>1.539296883</c:v>
+                </c:pt>
+                <c:pt idx="119">
+                  <c:v>1.544342546</c:v>
+                </c:pt>
+                <c:pt idx="120">
+                  <c:v>1.5493136649999999</c:v>
+                </c:pt>
+                <c:pt idx="121">
+                  <c:v>1.554218452</c:v>
+                </c:pt>
+                <c:pt idx="122">
+                  <c:v>1.559065224</c:v>
+                </c:pt>
+                <c:pt idx="123">
+                  <c:v>1.56386249</c:v>
+                </c:pt>
+                <c:pt idx="124">
+                  <c:v>1.5686190289999999</c:v>
+                </c:pt>
+                <c:pt idx="125">
+                  <c:v>1.5733439899999999</c:v>
+                </c:pt>
+                <c:pt idx="126">
+                  <c:v>1.578047006</c:v>
+                </c:pt>
+                <c:pt idx="127">
+                  <c:v>1.58273833</c:v>
+                </c:pt>
+                <c:pt idx="128">
+                  <c:v>1.587429</c:v>
+                </c:pt>
+                <c:pt idx="129">
+                  <c:v>1.592131035</c:v>
+                </c:pt>
+                <c:pt idx="130">
+                  <c:v>1.596857682</c:v>
+                </c:pt>
+                <c:pt idx="131">
+                  <c:v>1.60162373</c:v>
+                </c:pt>
+                <c:pt idx="132">
+                  <c:v>1.6064459019999999</c:v>
+                </c:pt>
+                <c:pt idx="133">
+                  <c:v>1.61134336</c:v>
+                </c:pt>
+                <c:pt idx="134">
+                  <c:v>1.61633838</c:v>
+                </c:pt>
+                <c:pt idx="135">
+                  <c:v>1.6214572309999999</c:v>
+                </c:pt>
+                <c:pt idx="136">
+                  <c:v>1.626731385</c:v>
+                </c:pt>
+                <c:pt idx="137">
+                  <c:v>1.6321991680000001</c:v>
+                </c:pt>
+                <c:pt idx="138">
+                  <c:v>1.6379081019999999</c:v>
+                </c:pt>
+                <c:pt idx="139">
+                  <c:v>1.643918266</c:v>
+                </c:pt>
+                <c:pt idx="140">
+                  <c:v>1.6503072539999999</c:v>
+                </c:pt>
+                <c:pt idx="141">
+                  <c:v>1.6571777080000001</c:v>
+                </c:pt>
+                <c:pt idx="142">
+                  <c:v>1.6646690660000001</c:v>
+                </c:pt>
+                <c:pt idx="143">
+                  <c:v>1.6729764810000001</c:v>
+                </c:pt>
+                <c:pt idx="144">
+                  <c:v>1.682382187</c:v>
+                </c:pt>
+                <c:pt idx="145">
+                  <c:v>1.6933085109999999</c:v>
+                </c:pt>
+                <c:pt idx="146">
+                  <c:v>1.7064062250000001</c:v>
+                </c:pt>
+                <c:pt idx="147">
+                  <c:v>1.722682651</c:v>
+                </c:pt>
+                <c:pt idx="148">
+                  <c:v>1.7435617729999999</c:v>
+                </c:pt>
+                <c:pt idx="149">
+                  <c:v>1.7702195489999999</c:v>
+                </c:pt>
+                <c:pt idx="150">
+                  <c:v>1.8009563260000001</c:v>
+                </c:pt>
+                <c:pt idx="151">
+                  <c:v>1.830665802</c:v>
+                </c:pt>
+                <c:pt idx="152">
+                  <c:v>1.856770349</c:v>
+                </c:pt>
+                <c:pt idx="153">
+                  <c:v>1.8795104650000001</c:v>
+                </c:pt>
+                <c:pt idx="154">
+                  <c:v>1.899586244</c:v>
+                </c:pt>
+                <c:pt idx="155">
+                  <c:v>1.9175875760000001</c:v>
+                </c:pt>
+                <c:pt idx="156">
+                  <c:v>1.9339526950000001</c:v>
+                </c:pt>
+                <c:pt idx="157">
+                  <c:v>1.94900243</c:v>
+                </c:pt>
+                <c:pt idx="158">
+                  <c:v>1.9629749059999999</c:v>
+                </c:pt>
+                <c:pt idx="159">
+                  <c:v>1.976050715</c:v>
+                </c:pt>
+                <c:pt idx="160">
+                  <c:v>1.988369973</c:v>
+                </c:pt>
+                <c:pt idx="161">
+                  <c:v>2.0000438169999999</c:v>
+                </c:pt>
+                <c:pt idx="162">
+                  <c:v>2.0111622329999999</c:v>
+                </c:pt>
+                <c:pt idx="163">
+                  <c:v>2.0217995059999998</c:v>
+                </c:pt>
+                <c:pt idx="164">
+                  <c:v>2.0320180840000002</c:v>
+                </c:pt>
+                <c:pt idx="165">
+                  <c:v>2.0418713880000001</c:v>
+                </c:pt>
+                <c:pt idx="166">
+                  <c:v>2.0514059040000001</c:v>
+                </c:pt>
+                <c:pt idx="167">
+                  <c:v>2.0606627670000002</c:v>
+                </c:pt>
+                <c:pt idx="168">
+                  <c:v>2.069679013</c:v>
+                </c:pt>
+                <c:pt idx="169">
+                  <c:v>2.0784885709999998</c:v>
+                </c:pt>
+                <c:pt idx="170">
+                  <c:v>2.087123106</c:v>
+                </c:pt>
+                <c:pt idx="171">
+                  <c:v>2.095612735</c:v>
+                </c:pt>
+                <c:pt idx="172">
+                  <c:v>2.103986688</c:v>
+                </c:pt>
+                <c:pt idx="173">
+                  <c:v>2.1122739419999998</c:v>
+                </c:pt>
+                <c:pt idx="174">
+                  <c:v>2.1205038620000001</c:v>
+                </c:pt>
+                <c:pt idx="175">
+                  <c:v>2.1287068979999999</c:v>
+                </c:pt>
+                <c:pt idx="176">
+                  <c:v>2.1369153750000001</c:v>
+                </c:pt>
+                <c:pt idx="177">
+                  <c:v>2.145164447</c:v>
+                </c:pt>
+                <c:pt idx="178">
+                  <c:v>2.1534932960000002</c:v>
+                </c:pt>
+                <c:pt idx="179">
+                  <c:v>2.1619466969999999</c:v>
+                </c:pt>
+                <c:pt idx="180">
+                  <c:v>2.170577142</c:v>
+                </c:pt>
+                <c:pt idx="181">
+                  <c:v>2.1794478239999999</c:v>
+                </c:pt>
+                <c:pt idx="182">
+                  <c:v>2.1886369779999999</c:v>
+                </c:pt>
+                <c:pt idx="183">
+                  <c:v>2.198244442</c:v>
+                </c:pt>
+                <c:pt idx="184">
+                  <c:v>2.2084020099999999</c:v>
+                </c:pt>
+                <c:pt idx="185">
+                  <c:v>2.2192906109999999</c:v>
+                </c:pt>
+                <c:pt idx="186">
+                  <c:v>2.2311706550000001</c:v>
+                </c:pt>
+                <c:pt idx="187">
+                  <c:v>2.244440011</c:v>
+                </c:pt>
+                <c:pt idx="188">
+                  <c:v>2.259756984</c:v>
+                </c:pt>
+                <c:pt idx="189">
+                  <c:v>2.2783425070000001</c:v>
+                </c:pt>
+                <c:pt idx="190">
+                  <c:v>2.302910223</c:v>
+                </c:pt>
+                <c:pt idx="191">
+                  <c:v>2.3396146099999999</c:v>
+                </c:pt>
+                <c:pt idx="192">
+                  <c:v>2.3943824020000002</c:v>
+                </c:pt>
+                <c:pt idx="193">
+                  <c:v>2.4770564140000002</c:v>
+                </c:pt>
+                <c:pt idx="194">
+                  <c:v>2.549458274</c:v>
+                </c:pt>
+                <c:pt idx="195">
+                  <c:v>2.6129149439999999</c:v>
+                </c:pt>
+                <c:pt idx="196">
+                  <c:v>2.6739977000000001</c:v>
+                </c:pt>
+                <c:pt idx="197">
+                  <c:v>2.7347374019999999</c:v>
+                </c:pt>
+                <c:pt idx="198">
+                  <c:v>2.7961824970000002</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-B90D-41A7-B9B0-D2E2F7482819}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="313001488"/>
+        <c:axId val="313004368"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="313001488"/>
+        <c:scaling>
+          <c:logBase val="10"/>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="da-DK"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="313004368"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="313004368"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="da-DK"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="313001488"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="da-DK"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>518160</xdr:colOff>
+      <xdr:row>183</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>213360</xdr:colOff>
+      <xdr:row>198</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Diagram 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AE3F8750-F30E-2845-C396-BD3556F48C12}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -500,12 +2641,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H203"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="5" width="17.85546875" customWidth="1"/>
+    <col min="4" max="5" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>9</v>
       </c>
@@ -516,7 +2657,7 @@
       <c r="F1" s="11"/>
       <c r="G1" s="11"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -533,7 +2674,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -550,7 +2691,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>0</v>
       </c>
@@ -567,7 +2708,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>6.8671679320000001</v>
       </c>
@@ -596,7 +2737,7 @@
         <v>0.21</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>13.05931629</v>
       </c>
@@ -625,7 +2766,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>18.550231419999999</v>
       </c>
@@ -654,7 +2795,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>23.4909325</v>
       </c>
@@ -683,7 +2824,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>27.986195899999998</v>
       </c>
@@ -712,7 +2853,7 @@
         <v>1.54</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>32.116098409999999</v>
       </c>
@@ -741,7 +2882,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>35.941569080000001</v>
       </c>
@@ -770,7 +2911,7 @@
         <v>2.65</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>39.509859179999999</v>
       </c>
@@ -799,7 +2940,7 @@
         <v>3.33</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>42.858295310000003</v>
       </c>
@@ -828,7 +2969,7 @@
         <v>4.05</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>46.016877360000002</v>
       </c>
@@ -857,7 +2998,7 @@
         <v>4.88</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>49.010094979999998</v>
       </c>
@@ -886,7 +3027,7 @@
         <v>5.79</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>51.8582204</v>
       </c>
@@ -915,7 +3056,7 @@
         <v>6.71</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>54.578245819999999</v>
       </c>
@@ -944,7 +3085,7 @@
         <v>7.73</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>57.184575760000001</v>
       </c>
@@ -973,7 +3114,7 @@
         <v>8.89</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>59.68954695</v>
       </c>
@@ -1002,7 +3143,7 @@
         <v>10.15</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>62.10382508</v>
       </c>
@@ -1031,7 +3172,7 @@
         <v>11.26</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>64.436711790000004</v>
       </c>
@@ -1060,7 +3201,7 @@
         <v>12.42</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>66.696385500000005</v>
       </c>
@@ -1080,7 +3221,7 @@
         <v>1794.0859544080843</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>68.89009265</v>
       </c>
@@ -1100,7 +3241,7 @@
         <v>1824.4753421122232</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>71.024301269999995</v>
       </c>
@@ -1120,7 +3261,7 @@
         <v>1854.5771631454734</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>73.10482571</v>
       </c>
@@ -1140,7 +3281,7 @@
         <v>1884.4164463265263</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>75.13692897</v>
       </c>
@@ -1160,7 +3301,7 @@
         <v>1914.0157786259701</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>77.125407510000002</v>
       </c>
@@ -1180,7 +3321,7 @@
         <v>1943.3955882787091</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>79.074662200000006</v>
       </c>
@@ -1200,7 +3341,7 @@
         <v>1972.574469276143</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>80.988758379999993</v>
       </c>
@@ -1220,7 +3361,7 @@
         <v>2001.5692627130306</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>82.871477060000004</v>
       </c>
@@ -1240,7 +3381,7 @@
         <v>2030.3953365464242</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>84.726359160000001</v>
       </c>
@@ -1260,7 +3401,7 @@
         <v>2059.0666317470827</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>86.556744080000001</v>
       </c>
@@ -1280,7 +3421,7 @@
         <v>2087.5957967083204</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <v>88.365803830000004</v>
       </c>
@@ -1300,7 +3441,7 @@
         <v>2115.9942597104382</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <v>90.156573429999995</v>
       </c>
@@ -1320,7 +3461,7 @@
         <v>2144.2723073601746</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <v>91.931978580000006</v>
       </c>
@@ -1340,7 +3481,7 @@
         <v>2172.439052234939</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
         <v>93.694861029999998</v>
       </c>
@@ -1360,7 +3501,7 @@
         <v>2200.5025152152134</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
         <v>95.448002320000001</v>
       </c>
@@ -1380,7 +3521,7 @@
         <v>2228.4695489063838</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>97.194146329999995</v>
       </c>
@@ -1400,7 +3541,7 @@
         <v>2256.3458547556816</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
         <v>98.936020979999995</v>
       </c>
@@ -1420,7 +3561,7 @@
         <v>2284.1359014877507</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>100.6763596</v>
       </c>
@@ -1440,7 +3581,7 @@
         <v>2311.8428192546526</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <v>102.4179221</v>
       </c>
@@ -1460,7 +3601,7 @@
         <v>2339.4683414755</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <v>104.16351659999999</v>
       </c>
@@ -1480,7 +3621,7 @@
         <v>2367.0125923641499</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
         <v>105.9160217</v>
       </c>
@@ -1500,7 +3641,7 @@
         <v>2394.4739601425958</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
         <v>107.6784092</v>
       </c>
@@ -1520,7 +3661,7 @@
         <v>2421.848829577109</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
         <v>109.4537684</v>
       </c>
@@ -1540,7 +3681,7 @@
         <v>2449.1313040727741</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
         <v>111.2453318</v>
       </c>
@@ -1560,7 +3701,7 @@
         <v>2476.3128798115531</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
         <v>113.05650249999999</v>
       </c>
@@ -1580,7 +3721,7 @@
         <v>2503.3820366972786</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
         <v>114.890883</v>
       </c>
@@ -1600,7 +3741,7 @@
         <v>2530.323715222411</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
         <v>116.752307</v>
       </c>
@@ -1620,7 +3761,7 @@
         <v>2557.1187286594077</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
         <v>118.64487219999999</v>
       </c>
@@ -1640,7 +3781,7 @@
         <v>2583.7430502528991</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
         <v>120.5729759</v>
       </c>
@@ -1660,7 +3801,7 @@
         <v>2610.1669651984935</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
         <v>122.54185200000001</v>
       </c>
@@ -1680,7 +3821,7 @@
         <v>2636.3608851894119</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
         <v>124.5896113</v>
       </c>
@@ -1700,7 +3841,7 @@
         <v>2662.7235121178956</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
         <v>126.7346713</v>
       </c>
@@ -1720,7 +3861,7 @@
         <v>2689.3896536404454</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
         <v>128.98503880000001</v>
       </c>
@@ -1740,7 +3881,7 @@
         <v>2716.3419549102891</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
         <v>131.34940180000001</v>
       </c>
@@ -1760,7 +3901,7 @@
         <v>2743.5538845100677</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="2">
         <v>133.83751520000001</v>
       </c>
@@ -1780,7 +3921,7 @@
         <v>2770.9915581280866</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
         <v>136.4603764</v>
       </c>
@@ -1800,7 +3941,7 @@
         <v>2798.6120929204494</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="2">
         <v>139.2304245</v>
       </c>
@@ -1820,7 +3961,7 @@
         <v>2826.3614661657921</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
         <v>142.16177329999999</v>
       </c>
@@ -1840,7 +3981,7 @@
         <v>2854.1718641491593</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
         <v>145.27047970000001</v>
       </c>
@@ -1860,7 +4001,7 @@
         <v>2881.9582998258447</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="2">
         <v>148.5748523</v>
       </c>
@@ -1880,7 +4021,7 @@
         <v>2909.6144366796862</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
         <v>152.0957946</v>
       </c>
@@ -1900,7 +4041,7 @@
         <v>2937.007362722793</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
         <v>155.8571772</v>
       </c>
@@ -1920,7 +4061,7 @@
         <v>2963.9711170559831</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
         <v>159.88621560000001</v>
       </c>
@@ -1940,7 +4081,7 @@
         <v>2990.2988370983862</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
         <v>164.2138118</v>
       </c>
@@ -1960,7 +4101,7 @@
         <v>3015.733416991005</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
         <v>168.87478369999999</v>
       </c>
@@ -1980,7 +4121,7 @@
         <v>3039.956877103742</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="2">
         <v>173.90785500000001</v>
       </c>
@@ -2000,7 +4141,7 @@
         <v>3062.5790220527019</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="2">
         <v>179.35520729999999</v>
       </c>
@@ -2020,7 +4161,7 @@
         <v>3083.127039766156</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="2">
         <v>185.26131860000001</v>
       </c>
@@ -2040,7 +4181,7 @@
         <v>3101.0388514112378</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="2">
         <v>191.67074589999999</v>
       </c>
@@ -2060,7 +4201,7 @@
         <v>3115.6651424898796</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="2">
         <v>198.62454410000001</v>
       </c>
@@ -2080,7 +4221,7 @@
         <v>3126.2868494588784</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="2">
         <v>206.15524479999999</v>
       </c>
@@ -2100,7 +4241,7 @@
         <v>3132.155814050102</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="2">
         <v>214.28088579999999</v>
       </c>
@@ -2120,7 +4261,7 @@
         <v>3132.5632050687486</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="2">
         <v>222.999425</v>
       </c>
@@ -2140,7 +4281,7 @@
         <v>3126.9315387440988</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="2">
         <v>232.2856074</v>
       </c>
@@ -2160,7 +4301,7 @@
         <v>3114.9117771101396</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" s="2">
         <v>242.09221479999999</v>
       </c>
@@ -2180,7 +4321,7 @@
         <v>3096.454940886927</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="2">
         <v>252.35615870000001</v>
       </c>
@@ -2200,7 +4341,7 @@
         <v>3071.8294228764717</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" s="2">
         <v>263.00770269999998</v>
       </c>
@@ -2220,7 +4361,7 @@
         <v>3041.5753728653926</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" s="2">
         <v>273.97977300000002</v>
       </c>
@@ -2240,7 +4381,7 @@
         <v>3006.4142187482971</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="2">
         <v>285.2147683</v>
       </c>
@@ -2260,7 +4401,7 @@
         <v>2967.1462086401407</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="2">
         <v>296.66790630000003</v>
       </c>
@@ -2280,7 +4421,7 @@
         <v>2924.5641420543084</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="2">
         <v>308.30761890000002</v>
       </c>
@@ -2300,7 +4441,7 @@
         <v>2879.3963616666556</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="2">
         <v>320.11414000000002</v>
       </c>
@@ -2320,7 +4461,7 @@
         <v>2832.2782265747378</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="2">
         <v>332.07734420000003</v>
       </c>
@@ -2340,7 +4481,7 @@
         <v>2783.7446560943599</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="2">
         <v>344.19452960000001</v>
       </c>
@@ -2360,7 +4501,7 @@
         <v>2734.2352531455217</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="2">
         <v>356.4684853</v>
       </c>
@@ -2380,7 +4521,7 @@
         <v>2684.1055059076884</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" s="2">
         <v>368.9059537</v>
       </c>
@@ -2400,7 +4541,7 @@
         <v>2633.6398088129449</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" s="2">
         <v>381.5164734</v>
       </c>
@@ -2420,7 +4561,7 @@
         <v>2583.064092080243</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" s="2">
         <v>394.31154479999998</v>
       </c>
@@ -2440,7 +4581,7 @@
         <v>2532.5569848222422</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" s="2">
         <v>407.30404549999997</v>
       </c>
@@ -2460,7 +4601,7 @@
         <v>2482.2592295651875</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" s="2">
         <v>420.50783389999998</v>
       </c>
@@ -2480,7 +4621,7 @@
         <v>2432.2813674401582</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" s="2">
         <v>433.93749050000002</v>
       </c>
@@ -2500,7 +4641,7 @@
         <v>2382.7099182817528</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" s="2">
         <v>447.60815580000002</v>
       </c>
@@ -2520,7 +4661,7 @@
         <v>2333.6123080585185</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" s="2">
         <v>461.53543960000002</v>
       </c>
@@ -2540,7 +4681,7 @@
         <v>2285.0407398011848</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="2">
         <v>475.73537870000001</v>
       </c>
@@ -2560,7 +4701,7 @@
         <v>2237.0352669239014</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" s="2">
         <v>490.22443070000003</v>
       </c>
@@ -2580,7 +4721,7 @@
         <v>2189.6262142430451</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" s="2">
         <v>505.0194932</v>
       </c>
@@ -2600,7 +4741,7 @@
         <v>2142.8360828696577</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" s="2">
         <v>520.13794180000002</v>
       </c>
@@ -2620,7 +4761,7 @@
         <v>2096.6810599335258</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" s="2">
         <v>535.59768250000002</v>
       </c>
@@ -2640,7 +4781,7 @@
         <v>2051.1722148213421</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101" s="2">
         <v>551.41721600000005</v>
       </c>
@@ -2660,7 +4801,7 @@
         <v>2006.3164545437464</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A102" s="2">
         <v>567.61571140000001</v>
       </c>
@@ -2680,7 +4821,7 @@
         <v>1962.1172831058491</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A103" s="2">
         <v>584.21308929999998</v>
       </c>
@@ -2700,7 +4841,7 @@
         <v>1918.5754112896127</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A104" s="2">
         <v>601.23011359999998</v>
       </c>
@@ -2720,7 +4861,7 @@
         <v>1875.6892437714901</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A105" s="2">
         <v>618.68849230000001</v>
       </c>
@@ -2740,7 +4881,7 @@
         <v>1833.4552742200608</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A106" s="2">
         <v>636.61098800000002</v>
       </c>
@@ -2760,7 +4901,7 @@
         <v>1791.8684025107334</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107" s="2">
         <v>655.02153920000001</v>
       </c>
@@ -2780,7 +4921,7 @@
         <v>1750.9221925721627</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A108" s="2">
         <v>673.94539320000001</v>
       </c>
@@ -2800,7 +4941,7 @@
         <v>1710.6090791149034</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A109" s="2">
         <v>693.4092531</v>
       </c>
@@ -2820,7 +4961,7 @@
         <v>1670.9205368608013</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110" s="2">
         <v>713.44144019999999</v>
       </c>
@@ -2840,7 +4981,7 @@
         <v>1631.8472194281203</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A111" s="2">
         <v>734.07207370000003</v>
       </c>
@@ -2860,7 +5001,7 @@
         <v>1593.3790664837984</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A112" s="2">
         <v>755.33327199999997</v>
       </c>
@@ -2880,7 +5021,7 @@
         <v>1555.5053888935927</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A113" s="2">
         <v>777.25937720000002</v>
       </c>
@@ -2900,7 +5041,7 @@
         <v>1518.2149456304724</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A114" s="2">
         <v>799.88720709999996</v>
       </c>
@@ -2920,7 +5061,7 @@
         <v>1481.4959929168433</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A115" s="2">
         <v>823.25634049999996</v>
       </c>
@@ -2940,7 +5081,7 @@
         <v>1445.3363249769029</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A116" s="2">
         <v>847.4094384</v>
       </c>
@@ -2960,7 +5101,7 @@
         <v>1409.7233063997244</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A117" s="2">
         <v>872.39261080000006</v>
       </c>
@@ -2980,7 +5121,7 @@
         <v>1374.6438892357821</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A118" s="2">
         <v>898.25583410000002</v>
       </c>
@@ -3000,7 +5141,7 @@
         <v>1340.0846255960619</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A119" s="2">
         <v>925.05342910000002</v>
       </c>
@@ -3020,7 +5161,7 @@
         <v>1306.0316663939477</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A120" s="2">
         <v>952.84461229999999</v>
       </c>
@@ -3040,7 +5181,7 @@
         <v>1272.4707563868137</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A121" s="2">
         <v>981.69413059999999</v>
       </c>
@@ -3060,7 +5201,7 @@
         <v>1239.3872197257065</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A122" s="2">
         <v>1011.672999</v>
       </c>
@@ -3080,7 +5221,7 @@
         <v>1206.7659359276947</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A123" s="2">
         <v>1042.859361</v>
       </c>
@@ -3100,7 +5241,7 @@
         <v>1174.5913062547504</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A124" s="2">
         <v>1075.3394949999999</v>
       </c>
@@ -3120,7 +5261,7 @@
         <v>1142.8472178594293</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A125" s="2">
         <v>1109.208995</v>
       </c>
@@ -3140,7 +5281,7 @@
         <v>1111.5169877637477</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A126" s="2">
         <v>1144.574179</v>
       </c>
@@ -3160,7 +5301,7 @@
         <v>1080.583302589223</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A127" s="2">
         <v>1181.55375</v>
       </c>
@@ -3180,7 +5321,7 @@
         <v>1050.0281388056746</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A128" s="2">
         <v>1220.280796</v>
       </c>
@@ -3200,7 +5341,7 @@
         <v>1019.8326746408117</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A129" s="2">
         <v>1260.905188</v>
       </c>
@@ -3220,7 +5361,7 @@
         <v>989.97717936806168</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A130" s="2">
         <v>1303.5964959999999</v>
       </c>
@@ -3240,7 +5381,7 @@
         <v>960.44088013729038</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A131" s="2">
         <v>1348.54755</v>
       </c>
@@ -3260,7 +5401,7 @@
         <v>931.20180091634813</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A132" s="2">
         <v>1395.9788100000001</v>
       </c>
@@ -3280,7 +5421,7 @@
         <v>902.23657779057339</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A133" s="2">
         <v>1446.1438089999999</v>
       </c>
@@ -3300,7 +5441,7 @@
         <v>873.52022179636606</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A134" s="2">
         <v>1499.3359479999999</v>
       </c>
@@ -3320,7 +5461,7 @@
         <v>845.02584163434415</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A135" s="2">
         <v>1555.8971039999999</v>
       </c>
@@ -3340,7 +5481,7 @@
         <v>816.72429639205086</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A136" s="2">
         <v>1616.228625</v>
       </c>
@@ -3360,7 +5501,7 @@
         <v>788.58377354496849</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A137" s="2">
         <v>1680.805537</v>
       </c>
@@ -3380,7 +5521,7 @@
         <v>760.56926421530011</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A138" s="2">
         <v>1750.1951570000001</v>
       </c>
@@ -3400,7 +5541,7 @@
         <v>732.64189920936747</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A139" s="2">
         <v>1825.0817930000001</v>
       </c>
@@ -3420,7 +5561,7 @@
         <v>704.75812063001138</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A140" s="2">
         <v>1906.3000460000001</v>
       </c>
@@ -3440,7 +5581,7 @@
         <v>676.86861222933419</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A141" s="2">
         <v>1994.8804689999999</v>
       </c>
@@ -3460,7 +5601,7 @@
         <v>648.91692767752272</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A142" s="2">
         <v>2092.1133540000001</v>
       </c>
@@ -3480,7 +5621,7 @@
         <v>620.83769314174299</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A143" s="2">
         <v>2199.6397459999998</v>
       </c>
@@ -3500,7 +5641,7 @@
         <v>592.55423811469052</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A144" s="2">
         <v>2319.5843589999999</v>
       </c>
@@ -3520,7 +5661,7 @@
         <v>563.97543175742123</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A145" s="2">
         <v>2454.75486</v>
       </c>
@@ -3540,7 +5681,7 @@
         <v>534.99141884683354</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A146" s="2">
         <v>2608.9495069999998</v>
       </c>
@@ -3560,7 +5701,7 @@
         <v>505.46785804447836</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A147" s="2">
         <v>2787.4477310000002</v>
       </c>
@@ -3580,7 +5721,7 @@
         <v>475.23816773242407</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A148" s="2">
         <v>2997.820471</v>
       </c>
@@ -3600,7 +5741,7 @@
         <v>444.09343255104204</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A149" s="2">
         <v>3251.318327</v>
       </c>
@@ -3620,7 +5761,7 @@
         <v>411.77057165895184</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A150" s="2">
         <v>3565.3275440000002</v>
       </c>
@@ -3640,7 +5781,7 @@
         <v>377.94342368173028</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A151" s="2">
         <v>3967.7694329999999</v>
       </c>
@@ -3660,7 +5801,7 @@
         <v>342.23634994106646</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A152" s="2">
         <v>4504.5108710000004</v>
       </c>
@@ -3680,7 +5821,7 @@
         <v>304.33210967524423</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A153" s="2">
         <v>5247.5704539999997</v>
       </c>
@@ -3700,7 +5841,7 @@
         <v>264.4047156598873</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A154" s="2">
         <v>6279.0885420000004</v>
       </c>
@@ -3720,7 +5861,7 @@
         <v>224.34720397454112</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A155" s="2">
         <v>7581.555816</v>
       </c>
@@ -3740,7 +5881,7 @@
         <v>189.031848166716</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A156" s="2">
         <v>8963.1991959999996</v>
       </c>
@@ -3760,7 +5901,7 @@
         <v>162.53098094016127</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A157" s="2">
         <v>10290.372460000001</v>
       </c>
@@ -3780,7 +5921,7 @@
         <v>143.58769829688634</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A158" s="2">
         <v>11547.06855</v>
       </c>
@@ -3800,7 +5941,7 @@
         <v>129.52784501209908</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A159" s="2">
         <v>12747.270490000001</v>
       </c>
@@ -3820,7 +5961,7 @@
         <v>118.58559869704592</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A160" s="2">
         <v>13907.195900000001</v>
       </c>
@@ -3840,7 +5981,7 @@
         <v>109.72504584191755</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A161" s="2">
         <v>15040.515219999999</v>
       </c>
@@ -3860,7 +6001,7 @@
         <v>102.32300111164099</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A162" s="2">
         <v>16158.14286</v>
       </c>
@@ -3880,7 +6021,7 @@
         <v>95.986702655200972</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A163" s="2">
         <v>17268.83959</v>
       </c>
@@ -3900,7 +6041,7 @@
         <v>90.456905869970086</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A164" s="2">
         <v>18379.815689999999</v>
       </c>
@@ -3920,7 +6061,7 @@
         <v>85.55532993283353</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A165" s="2">
         <v>19497.199700000001</v>
       </c>
@@ -3940,7 +6081,7 @@
         <v>81.154964499452817</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A166" s="2">
         <v>20626.38334</v>
       </c>
@@ -3960,7 +6101,7 @@
         <v>77.162548234675668</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A167" s="2">
         <v>21772.275300000001</v>
       </c>
@@ -3980,7 +6121,7 @@
         <v>73.507799789231058</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A168" s="2">
         <v>22939.492969999999</v>
       </c>
@@ -4000,7 +6141,7 @@
         <v>70.136551348687476</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A169" s="2">
         <v>24132.51296</v>
       </c>
@@ -4020,7 +6161,7 @@
         <v>67.006225803498381</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A170" s="2">
         <v>25355.795620000001</v>
       </c>
@@ -4040,7 +6181,7 @@
         <v>64.082770154090184</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A171" s="2">
         <v>26613.894390000001</v>
       </c>
@@ -4060,7 +6201,7 @@
         <v>61.33852211275309</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A172" s="2">
         <v>27911.557980000001</v>
       </c>
@@ -4080,7 +6221,7 @@
         <v>58.750691317280697</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A173" s="2">
         <v>29253.832170000001</v>
       </c>
@@ -4100,7 +6241,7 @@
         <v>56.300255573064135</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A174" s="2">
         <v>30646.166949999999</v>
       </c>
@@ -4120,7 +6261,7 @@
         <v>53.971142749168486</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A175" s="2">
         <v>32094.535100000001</v>
       </c>
@@ -4140,7 +6281,7 @@
         <v>51.749613777893579</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A176" s="2">
         <v>33605.568429999999</v>
       </c>
@@ -4160,7 +6301,7 @@
         <v>49.623788729583488</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A177" s="2">
         <v>35186.719559999998</v>
       </c>
@@ -4180,7 +6321,7 @@
         <v>47.583276557473063</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A178" s="2">
         <v>36846.459000000003</v>
       </c>
@@ -4200,7 +6341,7 @@
         <v>45.618880098288869</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A179" s="2">
         <v>38594.520369999998</v>
       </c>
@@ -4220,7 +6361,7 @@
         <v>43.722355951997841</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A180" s="2">
         <v>40442.211640000001</v>
       </c>
@@ -4240,7 +6381,7 @@
         <v>41.88621386811414</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A181" s="2">
         <v>42402.817309999999</v>
       </c>
@@ -4260,7 +6401,7 @@
         <v>40.103543405371099</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A182" s="2">
         <v>44492.127489999999</v>
       </c>
@@ -4280,7 +6421,7 @@
         <v>38.367857949901122</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A183" s="2">
         <v>46729.14718</v>
       </c>
@@ -4300,7 +6441,7 @@
         <v>36.672946507394201</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A184" s="2">
         <v>49137.066489999997</v>
       </c>
@@ -4320,7 +6461,7 @@
         <v>35.012723398818643</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A185" s="2">
         <v>51744.617610000001</v>
       </c>
@@ -4340,7 +6481,7 @@
         <v>33.381064298832186</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A186" s="2">
         <v>54588.021309999996</v>
       </c>
@@ -4360,7 +6501,7 @@
         <v>31.77161271615206</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A187" s="2">
         <v>57713.861089999999</v>
       </c>
@@ -4380,7 +6521,7 @@
         <v>30.177533360591848</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A188" s="2">
         <v>61183.473890000001</v>
       </c>
@@ -4400,7 +6541,7 @@
         <v>28.591173957986683</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A189" s="2">
         <v>65079.934569999998</v>
       </c>
@@ -4420,7 +6561,7 @@
         <v>27.003568653524635</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A190" s="2">
         <v>69519.727209999997</v>
       </c>
@@ -4440,7 +6581,7 @@
         <v>25.403657715106462</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A191" s="2">
         <v>74673.481299999999</v>
       </c>
@@ -4460,7 +6601,7 @@
         <v>23.776970916771216</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A192" s="2">
         <v>80805.828429999994</v>
       </c>
@@ -4480,7 +6621,7 @@
         <v>22.103215149469261</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A193" s="2">
         <v>88360.487080000006</v>
       </c>
@@ -4500,7 +6641,7 @@
         <v>20.351375715279332</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A194" s="2">
         <v>98170.869470000005</v>
       </c>
@@ -4520,7 +6661,7 @@
         <v>18.468282597631511</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A195" s="2">
         <v>112114.4518</v>
       </c>
@@ -4540,7 +6681,7 @@
         <v>16.345776106595967</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A196" s="2">
         <v>134675.64189999999</v>
       </c>
@@ -4560,7 +6701,7 @@
         <v>13.824371833623943</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A197" s="2">
         <v>171180.41440000001</v>
       </c>
@@ -4580,7 +6721,7 @@
         <v>11.13088189049698</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A198" s="2">
         <v>230246.37710000001</v>
       </c>
@@ -4600,7 +6741,7 @@
         <v>8.5611721142166104</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A199" s="2">
         <v>284156.97989999998</v>
       </c>
@@ -4620,7 +6761,7 @@
         <v>7.1396959289267796</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A200" s="2">
         <v>332357.217</v>
       </c>
@@ -4640,7 +6781,7 @@
         <v>6.2561952613817144</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A201" s="2">
         <v>379288.90899999999</v>
       </c>
@@ -4660,7 +6801,7 @@
         <v>5.6102345952246004</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A202" s="2">
         <v>426314.05430000002</v>
       </c>
@@ -4680,7 +6821,7 @@
         <v>5.1047692563321112</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A203" s="2">
         <v>474144.42190000002</v>
       </c>
@@ -4705,5 +6846,6 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>